<commit_message>
solved easy arrays 3 questions
</commit_message>
<xml_diff>
--- a/Questions.xlsx
+++ b/Questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shubham\Desktop\everything\GIt Work\Data_Structures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EB0532-0967-4DC7-A01F-BB061107CE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B99637-D455-4866-96A1-1ECAF3AA1D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="20">
   <si>
     <t>Sr no</t>
   </si>
@@ -64,6 +64,27 @@
   </si>
   <si>
     <t>Second largest</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Remove Duplicates</t>
+  </si>
+  <si>
+    <t>Leetcode</t>
+  </si>
+  <si>
+    <t>Array is Sorted</t>
+  </si>
+  <si>
+    <t>Missing number</t>
+  </si>
+  <si>
+    <t>Consecutives Ones</t>
   </si>
 </sst>
 </file>
@@ -384,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -451,6 +472,9 @@
       <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
@@ -467,6 +491,80 @@
       </c>
       <c r="E4" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>